<commit_message>
test(fixture): cover N/A and empty result in executed fixture (review feedback)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_tc_executed.xlsx
+++ b/tests/fixtures/sample_tc_executed.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -880,6 +880,90 @@
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="3" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>실행 샘플</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>1-9</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>샘플 케이스 9</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>1. 실행</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>정상</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>실행 샘플</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>샘플 케이스 10</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>1. 실행</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>정상</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>